<commit_message>
Image handoff: manifest of every placement, decisions without ERC photos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPK2bWpBHPAitKEehw7gcL
</commit_message>
<xml_diff>
--- a/docs/sfw-image-decisions-2026-10-05.xlsx
+++ b/docs/sfw-image-decisions-2026-10-05.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M143"/>
+  <dimension ref="A1:M146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1609,27 +1609,27 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Keep the photo, fix the link (card goes to localhost:8080).</t>
+          <t>Replace. Ecosystem Restoration Camps photos are dropped (Linnea, 5 Oct). Also fix the card link (goes to localhost:8080).</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>erc-rancho-cacachilas-agro8.jpg</t>
+          <t>hand-scooping-planter-bed-soil.jpg</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/erc-rancho-cacachilas-agro8.jpg</t>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/hand-scooping-planter-bed-soil.jpg</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Partner / graduate (permission needed)</t>
+          <t>Canva licence</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Aerial view of flowering crop rows and row covers</t>
+          <t>A hand lifting a scoop of dark crumbly soil from a planting bed</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1676,27 +1676,27 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Keep.</t>
+          <t>Replace. Ecosystem Restoration Camps photos are dropped (Linnea, 5 Oct).</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>erc-panchamana-treeplanting-2-fb-img-1666270988322.jpg</t>
+          <t>hvdb-inplanten-002.jpg</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/erc-panchamana-treeplanting-2-fb-img-1666270988322.jpg</t>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/hvdb-inplanten-002.jpg</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Partner / graduate (permission needed)</t>
+          <t>Owned (SFW archive). Photographer not recorded.</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Volunteers planting saplings in a eucalyptus forest</t>
+          <t>A group planting young trees across an open field on a grey day</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -1743,27 +1743,27 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Replace. forests.jpg is a 2020 upload with no record.</t>
+          <t>Replace. Ecosystem Restoration Camps photos are dropped (Linnea, 5 Oct).</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>erc-panchamana-garden.jpg</t>
+          <t>2-hands-planting-shrub.jpg</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/erc-panchamana-garden.jpg</t>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/2-hands-planting-shrub.jpg</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Partner / graduate (permission needed)</t>
+          <t>Canva licence</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Circular mandala vegetable garden from above</t>
+          <t>Two hands firming red soil around the base of a newly planted shrub</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>n/a, prototype has no such card</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1810,27 +1810,27 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Replace. Same treeplanting photo was on three cards.</t>
+          <t>Replace. Ecosystem Restoration Camps photos are dropped (Linnea, 5 Oct).</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>erc-panchamana-treeplanting-3-fb-img-1666271008784.jpg</t>
+          <t>2-hands-clasped-holding-plant-roots.jpg</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/erc-panchamana-treeplanting-3-fb-img-1666271008784.jpg</t>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/2-hands-clasped-holding-plant-roots.jpg</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Partner / graduate (permission needed)</t>
+          <t>Canva licence</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Volunteer crouching to plant a seedling</t>
+          <t>Weathered hands cupping a clump of loose soil around a young plant stem</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>n/a, prototype has no such card</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1877,27 +1877,27 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Replace. Same treeplanting photo was on three cards.</t>
+          <t>Replace. Ecosystem Restoration Camps photos are dropped (Linnea, 5 Oct).</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>erc-rancho-cacachilas-aerial-shot.jpg</t>
+          <t>fist-of-dry-soil.jpg</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/erc-rancho-cacachilas-aerial-shot.jpg</t>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/fist-of-dry-soil.jpg</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Partner / graduate (permission needed)</t>
+          <t>Canva licence</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Aerial view of desert scrub with mountains behind</t>
+          <t>A hand holding a clump of dry grey soil above more dry stony soil</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>n/a, prototype has no such card</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2511,27 +2511,27 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Replace. The four screenshots become the four photographs the prototype uses.</t>
+          <t>Replace. Ecosystem Restoration Camps photos are dropped (Linnea, 5 Oct).</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>erc-panchmana-treeplanting-fb-img-1666270907385.jpg</t>
+          <t>pile-turning-wes-8-scaled.jpg</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/erc-panchmana-treeplanting-fb-img-1666270907385.jpg</t>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/pile-turning-wes-8-scaled.jpg</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Partner / graduate (permission needed)</t>
+          <t>Owned (SFW archive). Photographer not recorded.</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Crowd of volunteers with potted seedlings in a forest clearing</t>
+          <t>Four people in gloves turning a compost pile by hand at a workshop</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr"/>
@@ -4403,27 +4403,27 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Keep the photo, fix the link (card goes to localhost:8080).</t>
+          <t>Replace. Ecosystem Restoration Camps photos are dropped (Linnea, 5 Oct). Also fix the card link (goes to localhost:8080).</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>erc-rancho-cacachilas-agro8.jpg</t>
+          <t>hand-scooping-planter-bed-soil.jpg</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/erc-rancho-cacachilas-agro8.jpg</t>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/hand-scooping-planter-bed-soil.jpg</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>Partner / graduate (permission needed)</t>
+          <t>Canva licence</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>Aerial view of flowering crop rows and row covers</t>
+          <t>A hand lifting a scoop of dark crumbly soil from a planting bed</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr">
@@ -4470,27 +4470,27 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Keep.</t>
+          <t>Replace. Ecosystem Restoration Camps photos are dropped (Linnea, 5 Oct).</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>erc-panchamana-treeplanting-2-fb-img-1666270988322.jpg</t>
+          <t>hvdb-inplanten-002.jpg</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/erc-panchamana-treeplanting-2-fb-img-1666270988322.jpg</t>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/hvdb-inplanten-002.jpg</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>Partner / graduate (permission needed)</t>
+          <t>Owned (SFW archive). Photographer not recorded.</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>Volunteers planting saplings in a eucalyptus forest</t>
+          <t>A group planting young trees across an open field on a grey day</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
@@ -4537,27 +4537,27 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Replace. forests.jpg is a 2020 upload with no record.</t>
+          <t>Replace. Ecosystem Restoration Camps photos are dropped (Linnea, 5 Oct).</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>erc-panchamana-garden.jpg</t>
+          <t>2-hands-planting-shrub.jpg</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/erc-panchamana-garden.jpg</t>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/2-hands-planting-shrub.jpg</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>Partner / graduate (permission needed)</t>
+          <t>Canva licence</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>Circular mandala vegetable garden from above</t>
+          <t>Two hands firming red soil around the base of a newly planted shrub</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">
@@ -4567,7 +4567,7 @@
       </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>n/a, prototype has no such card</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -4604,27 +4604,27 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Replace. Same treeplanting photo was on three cards.</t>
+          <t>Replace. Ecosystem Restoration Camps photos are dropped (Linnea, 5 Oct).</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>erc-panchamana-treeplanting-3-fb-img-1666271008784.jpg</t>
+          <t>2-hands-clasped-holding-plant-roots.jpg</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/erc-panchamana-treeplanting-3-fb-img-1666271008784.jpg</t>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/2-hands-clasped-holding-plant-roots.jpg</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>Partner / graduate (permission needed)</t>
+          <t>Canva licence</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>Volunteer crouching to plant a seedling</t>
+          <t>Weathered hands cupping a clump of loose soil around a young plant stem</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>n/a, prototype has no such card</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -4671,27 +4671,27 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Replace. Same treeplanting photo was on three cards.</t>
+          <t>Replace. Ecosystem Restoration Camps photos are dropped (Linnea, 5 Oct).</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>erc-rancho-cacachilas-aerial-shot.jpg</t>
+          <t>fist-of-dry-soil.jpg</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/erc-rancho-cacachilas-aerial-shot.jpg</t>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/fist-of-dry-soil.jpg</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>Partner / graduate (permission needed)</t>
+          <t>Canva licence</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>Aerial view of desert scrub with mountains behind</t>
+          <t>A hand holding a clump of dry grey soil above more dry stony soil</t>
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>n/a, prototype has no such card</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -8369,6 +8369,197 @@
       <c r="M143" s="2" t="inlineStr">
         <is>
           <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>community</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Workshop in Costa Rica, March 2025</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>(empty slot)</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Empty slot on staging</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Add.</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>costa-rica-2025-gerald-liquid-amendments.jpg</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/costa-rica-2025-gerald-liquid-amendments.jpg</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Owned (SFW drive, supplied 5 Oct)</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Mentor Gerald Ramirez, center, demonstrates how to make liquid amendments at our workshop in Costa Rica, March 2025</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>community</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Workshop in Costa Rica, March 2025</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>(empty slot)</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Empty slot on staging</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Add.</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>costa-rica-2025-microscopy-students-mentors.jpg</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/costa-rica-2025-microscopy-students-mentors.jpg</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Owned (SFW drive, supplied 5 Oct)</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Students and mentors practice microscopy together at our workshop in Costa Rica, March 2025</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>community</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Photo wall at the bottom of the page (new, 12 photos)</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Gallery</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>(new section)</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Linnea: a bunch of photos at the bottom of the community page</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Add. 3 by 4 grid, every photo 4:3, no captions.</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>cy-workshop-8.jpg, aug2023-workshop-group-7.jpg, pile-turning-wes-8-scaled.jpg, cy-classes-3.jpg, workshop-group-around-compost-pile.jpg, img-1942-scaled.jpg, cy-classes-4.jpg, ctpfw-student-moving-compost-1.jpg, elaine-ceremonial-compost-group-photo-scaled-1.jpg, ctpfw-student-squeezing-compost-1.jpg, elaine-flower-shirt-microscope.jpg, hand-of-compost.jpg</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>github.com/linneamoritznyc/final-SFWsite-Linnea/blob/claude/great-thompson-b408hm/img/</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Owned (SFW archive and SFW drive); hand-of-compost Canva licence</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>See community.html</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>Evan: which workshop and date for cy-workshop-8 and aug2023-workshop-group-7; confirm everyone pictured agreed to be published.</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>

</xml_diff>